<commit_message>
chore: update Homicidios dashboard — fresh data through May 2026
Regenerated via scripts/generate.py in himicidios-ecuador (live-browser
download bypassing the site's bot challenge). 35,460 records / 65 months.
</commit_message>
<xml_diff>
--- a/homicidios/provincias_stacked.xlsx
+++ b/homicidios/provincias_stacked.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mensual" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Mensual" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -804,7 +804,7 @@
         <v>19</v>
       </c>
       <c r="G11" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H11" t="n">
         <v>18</v>
@@ -813,7 +813,7 @@
         <v>82</v>
       </c>
       <c r="J11" t="n">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="12">
@@ -1218,10 +1218,10 @@
         <v>30</v>
       </c>
       <c r="I23" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J23" t="n">
-        <v>782</v>
+        <v>783</v>
       </c>
     </row>
     <row r="24">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C26" t="n">
         <v>96</v>
@@ -1320,10 +1320,10 @@
         <v>19</v>
       </c>
       <c r="I26" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J26" t="n">
-        <v>759</v>
+        <v>761</v>
       </c>
     </row>
     <row r="27">
@@ -1348,7 +1348,7 @@
         <v>25</v>
       </c>
       <c r="G27" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H27" t="n">
         <v>12</v>
@@ -1357,7 +1357,7 @@
         <v>64</v>
       </c>
       <c r="J27" t="n">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="28">
@@ -1388,10 +1388,10 @@
         <v>11</v>
       </c>
       <c r="I28" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J28" t="n">
-        <v>664</v>
+        <v>667</v>
       </c>
     </row>
     <row r="29">
@@ -1416,16 +1416,16 @@
         <v>29</v>
       </c>
       <c r="G29" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H29" t="n">
         <v>19</v>
       </c>
       <c r="I29" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J29" t="n">
-        <v>673</v>
+        <v>677</v>
       </c>
     </row>
     <row r="30">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>8610</v>
+        <v>8611</v>
       </c>
       <c r="C30" t="n">
         <v>2492</v>
@@ -1450,16 +1450,16 @@
         <v>765</v>
       </c>
       <c r="G30" t="n">
-        <v>705</v>
+        <v>710</v>
       </c>
       <c r="H30" t="n">
         <v>478</v>
       </c>
       <c r="I30" t="n">
-        <v>1891</v>
+        <v>1899</v>
       </c>
       <c r="J30" t="n">
-        <v>19121</v>
+        <v>19135</v>
       </c>
     </row>
   </sheetData>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8610</v>
+        <v>8611</v>
       </c>
       <c r="C2" t="n">
         <v>45</v>
@@ -1562,7 +1562,7 @@
         <v>1750</v>
       </c>
       <c r="C5" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>705</v>
+        <v>710</v>
       </c>
       <c r="C7" t="n">
         <v>3.7</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1891</v>
+        <v>1899</v>
       </c>
       <c r="C9" t="n">
         <v>9.9</v>

</xml_diff>

<commit_message>
data: update Homicidios Ecuador through 2026-06
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/homicidios/provincias_stacked.xlsx
+++ b/homicidios/provincias_stacked.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Mensual" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mensual" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1320,10 +1320,10 @@
         <v>19</v>
       </c>
       <c r="I26" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J26" t="n">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="27">
@@ -1456,10 +1456,10 @@
         <v>478</v>
       </c>
       <c r="I30" t="n">
-        <v>1899</v>
+        <v>1898</v>
       </c>
       <c r="J30" t="n">
-        <v>19135</v>
+        <v>19134</v>
       </c>
     </row>
   </sheetData>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1899</v>
+        <v>1898</v>
       </c>
       <c r="C9" t="n">
         <v>9.9</v>

</xml_diff>

<commit_message>
fix: make Homicidios 'Por Provincia' chart window roll forward automatically
The date range was hardcoded (Jan 2024-Apr 2026) in generate.py, so the
chart silently stopped updating past April even as fresh data landed.
Now derives a rolling 28-month window from the latest month in the data.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/homicidios/provincias_stacked.xlsx
+++ b/homicidios/provincias_stacked.xlsx
@@ -479,953 +479,953 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>260</v>
+        <v>232</v>
       </c>
       <c r="C2" t="n">
-        <v>43</v>
+        <v>100</v>
       </c>
       <c r="D2" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="G2" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H2" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="I2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J2" t="n">
-        <v>507</v>
+        <v>536</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="C3" t="n">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="D3" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E3" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F3" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G3" t="n">
+        <v>24</v>
+      </c>
+      <c r="H3" t="n">
         <v>13</v>
       </c>
-      <c r="H3" t="n">
-        <v>12</v>
-      </c>
       <c r="I3" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="J3" t="n">
-        <v>388</v>
+        <v>526</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="D4" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="F4" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G4" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="H4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I4" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J4" t="n">
-        <v>536</v>
+        <v>585</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2024-06</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="C5" t="n">
-        <v>79</v>
+        <v>45</v>
       </c>
       <c r="D5" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="F5" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="G5" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="H5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I5" t="n">
-        <v>49</v>
+        <v>89</v>
       </c>
       <c r="J5" t="n">
-        <v>526</v>
+        <v>611</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>241</v>
+        <v>266</v>
       </c>
       <c r="C6" t="n">
-        <v>112</v>
+        <v>44</v>
       </c>
       <c r="D6" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E6" t="n">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="F6" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="G6" t="n">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="H6" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="I6" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="J6" t="n">
-        <v>585</v>
+        <v>600</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>263</v>
+        <v>295</v>
       </c>
       <c r="C7" t="n">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="D7" t="n">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="E7" t="n">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="F7" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G7" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="H7" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I7" t="n">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="J7" t="n">
-        <v>611</v>
+        <v>621</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>266</v>
+        <v>304</v>
       </c>
       <c r="C8" t="n">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="D8" t="n">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="E8" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F8" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G8" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="H8" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I8" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="J8" t="n">
-        <v>600</v>
+        <v>610</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>295</v>
+        <v>320</v>
       </c>
       <c r="C9" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="D9" t="n">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="E9" t="n">
-        <v>52</v>
+        <v>90</v>
       </c>
       <c r="F9" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G9" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H9" t="n">
         <v>18</v>
       </c>
       <c r="I9" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="J9" t="n">
-        <v>621</v>
+        <v>701</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>304</v>
       </c>
       <c r="C10" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D10" t="n">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="E10" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F10" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="I10" t="n">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="J10" t="n">
-        <v>610</v>
+        <v>666</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>320</v>
+        <v>344</v>
       </c>
       <c r="C11" t="n">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D11" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E11" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="F11" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G11" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H11" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I11" t="n">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="J11" t="n">
-        <v>701</v>
+        <v>713</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>304</v>
+        <v>401</v>
       </c>
       <c r="C12" t="n">
-        <v>76</v>
+        <v>125</v>
       </c>
       <c r="D12" t="n">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="E12" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="F12" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G12" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H12" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="I12" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J12" t="n">
-        <v>666</v>
+        <v>800</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>344</v>
+        <v>391</v>
       </c>
       <c r="C13" t="n">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="D13" t="n">
-        <v>68</v>
+        <v>106</v>
       </c>
       <c r="E13" t="n">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="F13" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G13" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H13" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I13" t="n">
         <v>62</v>
       </c>
       <c r="J13" t="n">
-        <v>713</v>
+        <v>751</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>401</v>
+        <v>446</v>
       </c>
       <c r="C14" t="n">
-        <v>125</v>
+        <v>75</v>
       </c>
       <c r="D14" t="n">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="E14" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F14" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="G14" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="H14" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I14" t="n">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="J14" t="n">
-        <v>800</v>
+        <v>857</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>391</v>
+        <v>351</v>
       </c>
       <c r="C15" t="n">
-        <v>76</v>
+        <v>110</v>
       </c>
       <c r="D15" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E15" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F15" t="n">
+        <v>32</v>
+      </c>
+      <c r="G15" t="n">
         <v>31</v>
       </c>
-      <c r="G15" t="n">
-        <v>23</v>
-      </c>
       <c r="H15" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="I15" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="J15" t="n">
-        <v>751</v>
+        <v>742</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>446</v>
+        <v>469</v>
       </c>
       <c r="C16" t="n">
-        <v>75</v>
+        <v>119</v>
       </c>
       <c r="D16" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E16" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="F16" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="G16" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="H16" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I16" t="n">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="J16" t="n">
-        <v>857</v>
+        <v>935</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>351</v>
+        <v>247</v>
       </c>
       <c r="C17" t="n">
-        <v>110</v>
+        <v>69</v>
       </c>
       <c r="D17" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E17" t="n">
         <v>44</v>
       </c>
       <c r="F17" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G17" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H17" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I17" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="J17" t="n">
-        <v>742</v>
+        <v>574</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>469</v>
+        <v>255</v>
       </c>
       <c r="C18" t="n">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="D18" t="n">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="E18" t="n">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="F18" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G18" t="n">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="H18" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I18" t="n">
-        <v>93</v>
+        <v>55</v>
       </c>
       <c r="J18" t="n">
-        <v>935</v>
+        <v>637</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-08</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>247</v>
+        <v>291</v>
       </c>
       <c r="C19" t="n">
-        <v>69</v>
+        <v>130</v>
       </c>
       <c r="D19" t="n">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E19" t="n">
-        <v>44</v>
+        <v>87</v>
       </c>
       <c r="F19" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="G19" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="H19" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I19" t="n">
-        <v>40</v>
+        <v>97</v>
       </c>
       <c r="J19" t="n">
-        <v>574</v>
+        <v>771</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>255</v>
+        <v>319</v>
       </c>
       <c r="C20" t="n">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="D20" t="n">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="E20" t="n">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="F20" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="G20" t="n">
+        <v>21</v>
+      </c>
+      <c r="H20" t="n">
         <v>23</v>
       </c>
-      <c r="H20" t="n">
-        <v>21</v>
-      </c>
       <c r="I20" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="J20" t="n">
-        <v>637</v>
+        <v>771</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>291</v>
+        <v>278</v>
       </c>
       <c r="C21" t="n">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D21" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E21" t="n">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="F21" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="G21" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="H21" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="I21" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="J21" t="n">
-        <v>771</v>
+        <v>783</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>319</v>
+        <v>354</v>
       </c>
       <c r="C22" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D22" t="n">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="E22" t="n">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="F22" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G22" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="H22" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I22" t="n">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="J22" t="n">
-        <v>771</v>
+        <v>858</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>278</v>
+        <v>338</v>
       </c>
       <c r="C23" t="n">
-        <v>128</v>
+        <v>101</v>
       </c>
       <c r="D23" t="n">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="E23" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F23" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="G23" t="n">
         <v>31</v>
       </c>
       <c r="H23" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="I23" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J23" t="n">
-        <v>783</v>
+        <v>803</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>354</v>
+        <v>340</v>
       </c>
       <c r="C24" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>124</v>
+        <v>96</v>
       </c>
       <c r="E24" t="n">
-        <v>114</v>
+        <v>88</v>
       </c>
       <c r="F24" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="G24" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="H24" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I24" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="J24" t="n">
-        <v>858</v>
+        <v>760</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>338</v>
+        <v>299</v>
       </c>
       <c r="C25" t="n">
-        <v>101</v>
+        <v>76</v>
       </c>
       <c r="D25" t="n">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="E25" t="n">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="F25" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="G25" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="H25" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I25" t="n">
-        <v>94</v>
+        <v>64</v>
       </c>
       <c r="J25" t="n">
-        <v>803</v>
+        <v>684</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>340</v>
+        <v>301</v>
       </c>
       <c r="C26" t="n">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="D26" t="n">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="E26" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F26" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="G26" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H26" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="I26" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="J26" t="n">
-        <v>760</v>
+        <v>667</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>299</v>
+        <v>284</v>
       </c>
       <c r="C27" t="n">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="D27" t="n">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="E27" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="F27" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="G27" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H27" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="I27" t="n">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="J27" t="n">
-        <v>684</v>
+        <v>677</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="C28" t="n">
-        <v>71</v>
+        <v>123</v>
       </c>
       <c r="D28" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E28" t="n">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="F28" t="n">
         <v>27</v>
       </c>
       <c r="G28" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H28" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="I28" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J28" t="n">
-        <v>667</v>
+        <v>697</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>284</v>
+        <v>247</v>
       </c>
       <c r="C29" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D29" t="n">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="E29" t="n">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F29" t="n">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="G29" t="n">
         <v>19</v>
       </c>
       <c r="H29" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="I29" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J29" t="n">
-        <v>677</v>
+        <v>669</v>
       </c>
     </row>
     <row r="30">
@@ -1435,31 +1435,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>8611</v>
+        <v>8726</v>
       </c>
       <c r="C30" t="n">
-        <v>2492</v>
+        <v>2638</v>
       </c>
       <c r="D30" t="n">
-        <v>2430</v>
+        <v>2435</v>
       </c>
       <c r="E30" t="n">
-        <v>1750</v>
+        <v>1883</v>
       </c>
       <c r="F30" t="n">
-        <v>765</v>
+        <v>782</v>
       </c>
       <c r="G30" t="n">
-        <v>710</v>
+        <v>719</v>
       </c>
       <c r="H30" t="n">
-        <v>478</v>
+        <v>507</v>
       </c>
       <c r="I30" t="n">
-        <v>1898</v>
+        <v>1915</v>
       </c>
       <c r="J30" t="n">
-        <v>19134</v>
+        <v>19605</v>
       </c>
     </row>
   </sheetData>
@@ -1505,10 +1505,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8611</v>
+        <v>8726</v>
       </c>
       <c r="C2" t="n">
-        <v>45</v>
+        <v>44.5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2492</v>
+        <v>2638</v>
       </c>
       <c r="C3" t="n">
-        <v>13</v>
+        <v>13.5</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1541,10 +1541,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2430</v>
+        <v>2435</v>
       </c>
       <c r="C4" t="n">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1750</v>
+        <v>1883</v>
       </c>
       <c r="C5" t="n">
-        <v>9.1</v>
+        <v>9.6</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>765</v>
+        <v>782</v>
       </c>
       <c r="C6" t="n">
         <v>4</v>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>710</v>
+        <v>719</v>
       </c>
       <c r="C7" t="n">
         <v>3.7</v>
@@ -1613,10 +1613,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>478</v>
+        <v>507</v>
       </c>
       <c r="C8" t="n">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1631,10 +1631,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1898</v>
+        <v>1915</v>
       </c>
       <c r="C9" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>

</xml_diff>